<commit_message>
Project 3 Report JPG added
</commit_message>
<xml_diff>
--- a/TabularProject3/Docs and Final Reports/Countrywise Report for MyDatabase Project3.xlsx
+++ b/TabularProject3/Docs and Final Reports/Countrywise Report for MyDatabase Project3.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6447352ca101c75e/Desktop/ssas-learning/TabularProject3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6447352ca101c75e/Desktop/ssas-learning/TabularProject3/Docs and Final Reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D33A38F-DB43-4FE5-9921-5FD5E20F889B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{3D33A38F-DB43-4FE5-9921-5FD5E20F889B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31EEB03E-3872-4523-9DF0-500695BD0F9C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5ECF2E20-1C24-488A-8323-106583EBA480}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Countrywise Report" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="28" r:id="rId2"/>
+    <pivotCache cacheId="1" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -112,13 +112,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -216,7 +215,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A3D30E6-6F5E-4016-977A-30FDAD0C9FCA}" name="PivotTable4" cacheId="28" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A3D30E6-6F5E-4016-977A-30FDAD0C9FCA}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
   <location ref="A1:E5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -634,16 +633,16 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2">
         <v>350</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2">
         <v>500</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2">
         <v>425</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2">
         <v>850</v>
       </c>
     </row>
@@ -651,16 +650,16 @@
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3">
         <v>750</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3">
         <v>750</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3">
         <v>750</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3">
         <v>750</v>
       </c>
     </row>
@@ -668,16 +667,16 @@
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4">
         <v>0</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4">
         <v>900</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
         <v>450</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4">
         <v>900</v>
       </c>
     </row>
@@ -685,16 +684,16 @@
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>0</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5">
         <v>900</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5">
         <v>500</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5">
         <v>2500</v>
       </c>
     </row>

</xml_diff>